<commit_message>
Map closed Karelsky club to Rovio
</commit_message>
<xml_diff>
--- a/output/20260630_fix_owner_new_import/active_problem_3_non_named_payment_left_179_cases_20260630.xlsx
+++ b/output/20260630_fix_owner_new_import/active_problem_3_non_named_payment_left_179_cases_20260630.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>УТОЧНИТЬ: Карельский</t>
+          <t>Петрова Полина Владимировна</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="T84" s="2" t="inlineStr">
         <is>
-          <t>УТОЧНИТЬ: Карельский</t>
+          <t>Фёдорова Милана Андреевна</t>
         </is>
       </c>
     </row>

</xml_diff>